<commit_message>
commonName: A1#111DHARMAHEALTHCAREXX subject_application_id: HNRIS subject_application_vendor: DHARMA subject_application_version: 0.1
Aggiornati i file per l'accreditamento a seguito di vostra segnalazione di non conformità
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111DHARMAHEALTHCAREXX/DHARMA/HNRIS/0.1/accreditamento-checklist.xlsx
+++ b/GATEWAY/A1#111DHARMAHEALTHCAREXX/DHARMA/HNRIS/0.1/accreditamento-checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TMP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TMP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CBBBD9-089F-429A-9A91-F665576DF5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2380EAF-7300-4524-A9F2-F44C57AB5739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="193">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -793,15 +793,6 @@
   </si>
   <si>
     <t>5763a6f94262a8e4ab3845dca1a5cb38</t>
-  </si>
-  <si>
-    <t>9896e8eed83f6dc4274ee1e9063fc645</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.ecf37b5d8fd3845ab6b3d46859433fce51157db6d2fe127abe67f8a3c57f4b3b.006142b132^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2025-05-08T23:56:27Z</t>
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.120.4.4.99b609a8601241e42aebb05d2bcf1dfac8ab88afe6465521525ef7befd7d376c.15d730e8b3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
@@ -1412,6 +1403,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1446,9 +1440,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2923,14 +2914,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="47" t="s">
+      <c r="B2" s="47"/>
+      <c r="C2" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="D2" s="48"/>
+      <c r="D2" s="49"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -2951,14 +2942,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="55" t="s">
+      <c r="B3" s="51"/>
+      <c r="C3" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="48"/>
+      <c r="D3" s="49"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -2979,12 +2970,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="55" t="s">
+      <c r="A4" s="52"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="56" t="s">
         <v>141</v>
       </c>
-      <c r="D4" s="48"/>
+      <c r="D4" s="49"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -3006,12 +2997,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="53"/>
-      <c r="B5" s="54"/>
-      <c r="C5" s="55" t="s">
+      <c r="A5" s="54"/>
+      <c r="B5" s="55"/>
+      <c r="C5" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="48"/>
+      <c r="D5" s="49"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -3032,8 +3023,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="43"/>
-      <c r="B6" s="44"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="45"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -3188,10 +3179,10 @@
         <v>45786</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H10" s="33" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I10" s="37" t="s">
         <v>143</v>
@@ -3249,10 +3240,10 @@
         <v>45786</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I11" s="37" t="s">
         <v>143</v>
@@ -3712,7 +3703,7 @@
         <v>51</v>
       </c>
       <c r="O19" s="41" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="P19" s="29" t="s">
         <v>51</v>
@@ -3772,8 +3763,8 @@
       <c r="N20" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="O20" s="56" t="s">
-        <v>193</v>
+      <c r="O20" s="43" t="s">
+        <v>190</v>
       </c>
       <c r="P20" s="29" t="s">
         <v>51</v>
@@ -4199,22 +4190,16 @@
       <c r="E30" s="32" t="s">
         <v>105</v>
       </c>
-      <c r="F30" s="33">
-        <v>45785</v>
-      </c>
-      <c r="G30" s="33" t="s">
-        <v>185</v>
-      </c>
-      <c r="H30" s="33" t="s">
-        <v>183</v>
-      </c>
-      <c r="I30" s="37" t="s">
-        <v>184</v>
-      </c>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="37"/>
       <c r="J30" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="K30" s="29"/>
+        <v>83</v>
+      </c>
+      <c r="K30" s="29" t="s">
+        <v>88</v>
+      </c>
       <c r="L30" s="29"/>
       <c r="M30" s="29"/>
       <c r="N30" s="29"/>
@@ -4291,13 +4276,13 @@
         <v>45786</v>
       </c>
       <c r="G32" s="31" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H32" s="31" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="I32" s="29" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J32" s="31" t="s">
         <v>51</v>
@@ -4311,7 +4296,7 @@
         <v>51</v>
       </c>
       <c r="O32" s="29" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="P32" s="29" t="s">
         <v>51</v>
@@ -10719,6 +10704,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d4db60622090a1f8a8d506ac1d64a349">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a3a9ed8bb952a3d76dd1e2fa3d624b9" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -10976,28 +10982,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CE213DB-5082-48B0-B2A5-099EBF944035}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11014,29 +11024,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>